<commit_message>
Fixed table (25 -> 1000)
</commit_message>
<xml_diff>
--- a/prilohy/tabulky/projekty_cas.xlsx
+++ b/prilohy/tabulky/projekty_cas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cerny\Desktop\skola\Ekonomka\diplomka\zdroje\preciosa_zdroje\codex_source\prilohy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF10969-DD2E-4317-99A9-5CD4C895008F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7179E858-E8CC-4D58-988E-9DE3B70518B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{F6692C3A-DE33-40F4-869D-20D1512F99E5}"/>
   </bookViews>
@@ -1010,7 +1010,7 @@
         <v>32</v>
       </c>
       <c r="B3">
-        <v>25</v>
+        <v>1000</v>
       </c>
       <c r="C3" t="s">
         <v>33</v>

</xml_diff>